<commit_message>
chore(data-release): publish site data 2026-08-13 01:20:56 UTC
</commit_message>
<xml_diff>
--- a/countries/kr/2026-2029.xlsx
+++ b/countries/kr/2026-2029.xlsx
@@ -64130,16 +64130,16 @@
         </is>
       </c>
       <c r="N408" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O408" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q408" t="n">
         <v>0</v>
       </c>
       <c r="R408" t="n">
-        <v>0.003875939847584092</v>
+        <v>0.005813909771376137</v>
       </c>
       <c r="S408" t="inlineStr">
         <is>
@@ -66598,16 +66598,16 @@
         </is>
       </c>
       <c r="N424" t="n">
-        <v>5090</v>
+        <v>5089</v>
       </c>
       <c r="O424" t="n">
-        <v>5090</v>
+        <v>5089</v>
       </c>
       <c r="Q424" t="n">
         <v>0</v>
       </c>
       <c r="R424" t="n">
-        <v>9.864266912101515</v>
+        <v>9.862328942177722</v>
       </c>
       <c r="S424" t="inlineStr">
         <is>
@@ -66760,10 +66760,10 @@
         </is>
       </c>
       <c r="N425" t="n">
-        <v>5090</v>
+        <v>5089</v>
       </c>
       <c r="O425" t="n">
-        <v>5090</v>
+        <v>5089</v>
       </c>
       <c r="U425" t="inlineStr">
         <is>
@@ -68130,16 +68130,16 @@
         </is>
       </c>
       <c r="N433" t="n">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="O433" t="n">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="Q433" t="n">
         <v>0</v>
       </c>
       <c r="R433" t="n">
-        <v>0.8643345860112523</v>
+        <v>0.8604586461636684</v>
       </c>
       <c r="S433" t="inlineStr">
         <is>
@@ -71243,16 +71243,16 @@
         </is>
       </c>
       <c r="N452" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O452" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q452" t="n">
         <v>0</v>
       </c>
       <c r="R452" t="n">
-        <v>0.1627894735985319</v>
+        <v>0.1647274435223239</v>
       </c>
       <c r="S452" t="inlineStr">
         <is>
@@ -71391,16 +71391,16 @@
         </is>
       </c>
       <c r="N453" t="n">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="O453" t="n">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="Q453" t="n">
         <v>0</v>
       </c>
       <c r="R453" t="n">
-        <v>1.145340224961099</v>
+        <v>1.147278194884891</v>
       </c>
       <c r="S453" t="inlineStr">
         <is>
@@ -72575,16 +72575,16 @@
         </is>
       </c>
       <c r="N461" t="n">
-        <v>2508</v>
+        <v>2507</v>
       </c>
       <c r="O461" t="n">
-        <v>2508</v>
+        <v>2507</v>
       </c>
       <c r="Q461" t="n">
         <v>0</v>
       </c>
       <c r="R461" t="n">
-        <v>4.860428568870451</v>
+        <v>4.858490598946659</v>
       </c>
       <c r="S461" t="inlineStr">
         <is>
@@ -74051,16 +74051,16 @@
         </is>
       </c>
       <c r="N471" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O471" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q471" t="n">
         <v>0</v>
       </c>
       <c r="R471" t="n">
-        <v>0.1647274435223239</v>
+        <v>0.1666654134461159</v>
       </c>
       <c r="S471" t="inlineStr">
         <is>
@@ -77703,16 +77703,16 @@
         </is>
       </c>
       <c r="N495" t="n">
-        <v>5554</v>
+        <v>5553</v>
       </c>
       <c r="O495" t="n">
-        <v>5554</v>
+        <v>5553</v>
       </c>
       <c r="Q495" t="n">
         <v>0</v>
       </c>
       <c r="R495" t="n">
-        <v>10.76348495674102</v>
+        <v>10.76154698681723</v>
       </c>
       <c r="S495" t="inlineStr">
         <is>
@@ -77865,10 +77865,10 @@
         </is>
       </c>
       <c r="N496" t="n">
-        <v>5554</v>
+        <v>5553</v>
       </c>
       <c r="O496" t="n">
-        <v>5554</v>
+        <v>5553</v>
       </c>
       <c r="U496" t="inlineStr">
         <is>
@@ -78939,16 +78939,16 @@
         </is>
       </c>
       <c r="N502" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="O502" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="Q502" t="n">
         <v>0</v>
       </c>
       <c r="R502" t="n">
-        <v>0.0465112781710091</v>
+        <v>0.06976691725651366</v>
       </c>
       <c r="S502" t="inlineStr">
         <is>
@@ -79087,16 +79087,16 @@
         </is>
       </c>
       <c r="N503" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O503" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q503" t="n">
         <v>0</v>
       </c>
       <c r="R503" t="n">
-        <v>0.001937969923792046</v>
+        <v>0.003875939847584092</v>
       </c>
       <c r="S503" t="inlineStr">
         <is>
@@ -79235,16 +79235,16 @@
         </is>
       </c>
       <c r="N504" t="n">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="O504" t="n">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="Q504" t="n">
         <v>0</v>
       </c>
       <c r="R504" t="n">
-        <v>0.1860451126840364</v>
+        <v>0.2151146615409171</v>
       </c>
       <c r="S504" t="inlineStr">
         <is>
@@ -79383,16 +79383,16 @@
         </is>
       </c>
       <c r="N505" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O505" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q505" t="n">
         <v>0</v>
       </c>
       <c r="R505" t="n">
-        <v>0.01356578946654432</v>
+        <v>0.01744172931412841</v>
       </c>
       <c r="S505" t="inlineStr">
         <is>
@@ -80916,16 +80916,16 @@
         </is>
       </c>
       <c r="N514" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O514" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q514" t="n">
         <v>0</v>
       </c>
       <c r="R514" t="n">
-        <v>0.003875939847584092</v>
+        <v>0.007751879695168184</v>
       </c>
       <c r="S514" t="inlineStr">
         <is>
@@ -81212,16 +81212,16 @@
         </is>
       </c>
       <c r="N516" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="O516" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q516" t="n">
         <v>0</v>
       </c>
       <c r="R516" t="n">
-        <v>0.02713157893308864</v>
+        <v>0.02906954885688069</v>
       </c>
       <c r="S516" t="inlineStr">
         <is>
@@ -81508,16 +81508,16 @@
         </is>
       </c>
       <c r="N518" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O518" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Q518" t="n">
         <v>0</v>
       </c>
       <c r="R518" t="n">
-        <v>0.2422462404740058</v>
+        <v>0.2441842103977978</v>
       </c>
       <c r="S518" t="inlineStr">
         <is>
@@ -81804,16 +81804,16 @@
         </is>
       </c>
       <c r="N520" t="n">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="O520" t="n">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="Q520" t="n">
         <v>0</v>
       </c>
       <c r="R520" t="n">
-        <v>0.08527067664685002</v>
+        <v>0.09883646611339433</v>
       </c>
       <c r="S520" t="inlineStr">
         <is>
@@ -81966,10 +81966,10 @@
         </is>
       </c>
       <c r="N521" t="n">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="O521" t="n">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="U521" t="inlineStr">
         <is>
@@ -82348,16 +82348,16 @@
         </is>
       </c>
       <c r="N523" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="O523" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="Q523" t="n">
         <v>0</v>
       </c>
       <c r="R523" t="n">
-        <v>0.02713157893308864</v>
+        <v>0.03100751878067274</v>
       </c>
       <c r="S523" t="inlineStr">
         <is>
@@ -82496,16 +82496,16 @@
         </is>
       </c>
       <c r="N524" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="O524" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="Q524" t="n">
         <v>0</v>
       </c>
       <c r="R524" t="n">
-        <v>0.2422462404740058</v>
+        <v>0.2480601502453819</v>
       </c>
       <c r="S524" t="inlineStr">
         <is>
@@ -83680,16 +83680,16 @@
         </is>
       </c>
       <c r="N532" t="n">
-        <v>552</v>
+        <v>568</v>
       </c>
       <c r="O532" t="n">
-        <v>552</v>
+        <v>568</v>
       </c>
       <c r="Q532" t="n">
         <v>0</v>
       </c>
       <c r="R532" t="n">
-        <v>1.069759397933209</v>
+        <v>1.100766916713882</v>
       </c>
       <c r="S532" t="inlineStr">
         <is>
@@ -85156,16 +85156,16 @@
         </is>
       </c>
       <c r="N542" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="O542" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="Q542" t="n">
         <v>0</v>
       </c>
       <c r="R542" t="n">
-        <v>0.03294548870446478</v>
+        <v>0.04069736839963296</v>
       </c>
       <c r="S542" t="inlineStr">
         <is>
@@ -85748,16 +85748,16 @@
         </is>
       </c>
       <c r="N546" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O546" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q546" t="n">
         <v>0</v>
       </c>
       <c r="R546" t="n">
-        <v>0.01356578946654432</v>
+        <v>0.01744172931412841</v>
       </c>
       <c r="S546" t="inlineStr">
         <is>
@@ -86488,16 +86488,16 @@
         </is>
       </c>
       <c r="N551" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O551" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q551" t="n">
         <v>0</v>
       </c>
       <c r="R551" t="n">
-        <v>0.003875939847584092</v>
+        <v>0.005813909771376137</v>
       </c>
       <c r="S551" t="inlineStr">
         <is>
@@ -88808,16 +88808,16 @@
         </is>
       </c>
       <c r="N566" t="n">
-        <v>1827</v>
+        <v>1976</v>
       </c>
       <c r="O566" t="n">
-        <v>1827</v>
+        <v>1976</v>
       </c>
       <c r="Q566" t="n">
         <v>0</v>
       </c>
       <c r="R566" t="n">
-        <v>3.540671050768068</v>
+        <v>3.829428569413083</v>
       </c>
       <c r="S566" t="inlineStr">
         <is>
@@ -88970,10 +88970,10 @@
         </is>
       </c>
       <c r="N567" t="n">
-        <v>1827</v>
+        <v>1976</v>
       </c>
       <c r="O567" t="n">
-        <v>1827</v>
+        <v>1976</v>
       </c>
       <c r="U567" t="inlineStr">
         <is>
@@ -89711,7 +89711,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>74432</v>
+        <v>74649</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-15 02:00:33 UTC
</commit_message>
<xml_diff>
--- a/countries/kr/2026-2029.xlsx
+++ b/countries/kr/2026-2029.xlsx
@@ -55745,13 +55745,13 @@
         </is>
       </c>
       <c r="N360" t="n">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O360" t="n">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="R360" t="n">
-        <v>0.3837180449108251</v>
+        <v>0.3856560148346171</v>
       </c>
       <c r="S360" t="inlineStr">
         <is>
@@ -62431,13 +62431,13 @@
         </is>
       </c>
       <c r="N404" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O404" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="R404" t="n">
-        <v>0.2403082705502137</v>
+        <v>0.2422462404740058</v>
       </c>
       <c r="S404" t="inlineStr">
         <is>
@@ -65434,13 +65434,13 @@
         </is>
       </c>
       <c r="N424" t="n">
-        <v>5089</v>
+        <v>5087</v>
       </c>
       <c r="O424" t="n">
-        <v>5089</v>
+        <v>5087</v>
       </c>
       <c r="R424" t="n">
-        <v>9.862328942177722</v>
+        <v>9.858453002330137</v>
       </c>
       <c r="S424" t="inlineStr">
         <is>
@@ -65593,10 +65593,10 @@
         </is>
       </c>
       <c r="N425" t="n">
-        <v>5089</v>
+        <v>5087</v>
       </c>
       <c r="O425" t="n">
-        <v>5089</v>
+        <v>5087</v>
       </c>
       <c r="U425" t="inlineStr">
         <is>
@@ -73196,13 +73196,13 @@
         </is>
       </c>
       <c r="N474" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="O474" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="R474" t="n">
-        <v>0.01937969923792046</v>
+        <v>0.01744172931412841</v>
       </c>
       <c r="S474" t="inlineStr">
         <is>
@@ -73341,13 +73341,13 @@
         </is>
       </c>
       <c r="N475" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O475" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="R475" t="n">
-        <v>0.2732537592546785</v>
+        <v>0.2751917291784705</v>
       </c>
       <c r="S475" t="inlineStr">
         <is>
@@ -76344,13 +76344,13 @@
         </is>
       </c>
       <c r="N495" t="n">
-        <v>5552</v>
+        <v>5550</v>
       </c>
       <c r="O495" t="n">
-        <v>5552</v>
+        <v>5550</v>
       </c>
       <c r="R495" t="n">
-        <v>10.75960901689344</v>
+        <v>10.75573307704586</v>
       </c>
       <c r="S495" t="inlineStr">
         <is>
@@ -76503,10 +76503,10 @@
         </is>
       </c>
       <c r="N496" t="n">
-        <v>5552</v>
+        <v>5550</v>
       </c>
       <c r="O496" t="n">
-        <v>5552</v>
+        <v>5550</v>
       </c>
       <c r="U496" t="inlineStr">
         <is>
@@ -77565,13 +77565,13 @@
         </is>
       </c>
       <c r="N502" t="n">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="O502" t="n">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="R502" t="n">
-        <v>0.06976691725651366</v>
+        <v>0.09689849618960229</v>
       </c>
       <c r="S502" t="inlineStr">
         <is>
@@ -77855,13 +77855,13 @@
         </is>
       </c>
       <c r="N504" t="n">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="O504" t="n">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="R504" t="n">
-        <v>0.2868195487212228</v>
+        <v>0.294571428416391</v>
       </c>
       <c r="S504" t="inlineStr">
         <is>
@@ -78000,13 +78000,13 @@
         </is>
       </c>
       <c r="N505" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O505" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="R505" t="n">
-        <v>0.02325563908550455</v>
+        <v>0.02713157893308864</v>
       </c>
       <c r="S505" t="inlineStr">
         <is>
@@ -80092,13 +80092,13 @@
         </is>
       </c>
       <c r="N518" t="n">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="O518" t="n">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="R518" t="n">
-        <v>0.3003853381877671</v>
+        <v>0.3217030073494796</v>
       </c>
       <c r="S518" t="inlineStr">
         <is>
@@ -80382,13 +80382,13 @@
         </is>
       </c>
       <c r="N520" t="n">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="O520" t="n">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="R520" t="n">
-        <v>0.1027124059609784</v>
+        <v>0.1220921051988989</v>
       </c>
       <c r="S520" t="inlineStr">
         <is>
@@ -80541,10 +80541,10 @@
         </is>
       </c>
       <c r="N521" t="n">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="O521" t="n">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="U521" t="inlineStr">
         <is>
@@ -81065,13 +81065,13 @@
         </is>
       </c>
       <c r="N524" t="n">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="O524" t="n">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="R524" t="n">
-        <v>0.2984473682639751</v>
+        <v>0.3061992479591433</v>
       </c>
       <c r="S524" t="inlineStr">
         <is>
@@ -82225,13 +82225,13 @@
         </is>
       </c>
       <c r="N532" t="n">
-        <v>669</v>
+        <v>683</v>
       </c>
       <c r="O532" t="n">
-        <v>669</v>
+        <v>683</v>
       </c>
       <c r="R532" t="n">
-        <v>1.296501879016879</v>
+        <v>1.323633457949967</v>
       </c>
       <c r="S532" t="inlineStr">
         <is>
@@ -82515,13 +82515,13 @@
         </is>
       </c>
       <c r="N534" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O534" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R534" t="n">
-        <v>0.009689849618960231</v>
+        <v>0.01162781954275227</v>
       </c>
       <c r="S534" t="inlineStr">
         <is>
@@ -83526,13 +83526,13 @@
         </is>
       </c>
       <c r="N541" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O541" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R541" t="n">
-        <v>0.01744172931412841</v>
+        <v>0.01937969923792046</v>
       </c>
       <c r="S541" t="inlineStr">
         <is>
@@ -83816,13 +83816,13 @@
         </is>
       </c>
       <c r="N543" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O543" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R543" t="n">
-        <v>0.001937969923792046</v>
+        <v>0.005813909771376137</v>
       </c>
       <c r="S543" t="inlineStr">
         <is>
@@ -84251,13 +84251,13 @@
         </is>
       </c>
       <c r="N546" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="O546" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R546" t="n">
-        <v>0.01744172931412841</v>
+        <v>0.02131766916171251</v>
       </c>
       <c r="S546" t="inlineStr">
         <is>
@@ -87254,13 +87254,13 @@
         </is>
       </c>
       <c r="N566" t="n">
-        <v>2159</v>
+        <v>2341</v>
       </c>
       <c r="O566" t="n">
-        <v>2159</v>
+        <v>2341</v>
       </c>
       <c r="R566" t="n">
-        <v>4.184077065467028</v>
+        <v>4.53678759159718</v>
       </c>
       <c r="S566" t="inlineStr">
         <is>
@@ -87413,10 +87413,10 @@
         </is>
       </c>
       <c r="N567" t="n">
-        <v>2159</v>
+        <v>2341</v>
       </c>
       <c r="O567" t="n">
-        <v>2159</v>
+        <v>2341</v>
       </c>
       <c r="U567" t="inlineStr">
         <is>
@@ -88151,7 +88151,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>75058</v>
+        <v>75303</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-19 02:00:17 UTC
</commit_message>
<xml_diff>
--- a/countries/kr/2026-2029.xlsx
+++ b/countries/kr/2026-2029.xlsx
@@ -61561,13 +61561,13 @@
         </is>
       </c>
       <c r="N398" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O398" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R398" t="n">
-        <v>0.007751879695168184</v>
+        <v>0.009689849618960231</v>
       </c>
       <c r="S398" t="inlineStr">
         <is>
@@ -61996,13 +61996,13 @@
         </is>
       </c>
       <c r="N401" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O401" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R401" t="n">
-        <v>0.009689849618960231</v>
+        <v>0.007751879695168184</v>
       </c>
       <c r="S401" t="inlineStr">
         <is>
@@ -62431,13 +62431,13 @@
         </is>
       </c>
       <c r="N404" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O404" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="R404" t="n">
-        <v>0.2422462404740058</v>
+        <v>0.2441842103977978</v>
       </c>
       <c r="S404" t="inlineStr">
         <is>
@@ -65434,13 +65434,13 @@
         </is>
       </c>
       <c r="N424" t="n">
-        <v>5087</v>
+        <v>5082</v>
       </c>
       <c r="O424" t="n">
-        <v>5087</v>
+        <v>5082</v>
       </c>
       <c r="R424" t="n">
-        <v>9.858453002330137</v>
+        <v>9.848763152711177</v>
       </c>
       <c r="S424" t="inlineStr">
         <is>
@@ -65593,10 +65593,10 @@
         </is>
       </c>
       <c r="N425" t="n">
-        <v>5087</v>
+        <v>5082</v>
       </c>
       <c r="O425" t="n">
-        <v>5087</v>
+        <v>5082</v>
       </c>
       <c r="U425" t="inlineStr">
         <is>
@@ -69182,13 +69182,13 @@
         </is>
       </c>
       <c r="N447" t="n">
-        <v>852</v>
+        <v>855</v>
       </c>
       <c r="O447" t="n">
-        <v>852</v>
+        <v>855</v>
       </c>
       <c r="R447" t="n">
-        <v>1.651150375070823</v>
+        <v>1.656964284842199</v>
       </c>
       <c r="S447" t="inlineStr">
         <is>
@@ -70010,13 +70010,13 @@
         </is>
       </c>
       <c r="N452" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="O452" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="R452" t="n">
-        <v>0.1647274435223239</v>
+        <v>0.1608515036747398</v>
       </c>
       <c r="S452" t="inlineStr">
         <is>
@@ -71315,13 +71315,13 @@
         </is>
       </c>
       <c r="N461" t="n">
-        <v>2508</v>
+        <v>2509</v>
       </c>
       <c r="O461" t="n">
-        <v>2508</v>
+        <v>2509</v>
       </c>
       <c r="R461" t="n">
-        <v>4.860428568870451</v>
+        <v>4.862366538794243</v>
       </c>
       <c r="S461" t="inlineStr">
         <is>
@@ -72616,13 +72616,13 @@
         </is>
       </c>
       <c r="N470" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="O470" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="R470" t="n">
-        <v>0.04457330824721705</v>
+        <v>0.04844924809480115</v>
       </c>
       <c r="S470" t="inlineStr">
         <is>
@@ -72761,13 +72761,13 @@
         </is>
       </c>
       <c r="N471" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O471" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="R471" t="n">
-        <v>0.1705413532937</v>
+        <v>0.168603383369908</v>
       </c>
       <c r="S471" t="inlineStr">
         <is>
@@ -72906,13 +72906,13 @@
         </is>
       </c>
       <c r="N472" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O472" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R472" t="n">
-        <v>0.005813909771376137</v>
+        <v>0.003875939847584092</v>
       </c>
       <c r="S472" t="inlineStr">
         <is>
@@ -76344,13 +76344,13 @@
         </is>
       </c>
       <c r="N495" t="n">
-        <v>5550</v>
+        <v>5544</v>
       </c>
       <c r="O495" t="n">
-        <v>5550</v>
+        <v>5544</v>
       </c>
       <c r="R495" t="n">
-        <v>10.75573307704586</v>
+        <v>10.7441052575031</v>
       </c>
       <c r="S495" t="inlineStr">
         <is>
@@ -76503,10 +76503,10 @@
         </is>
       </c>
       <c r="N496" t="n">
-        <v>5550</v>
+        <v>5544</v>
       </c>
       <c r="O496" t="n">
-        <v>5550</v>
+        <v>5544</v>
       </c>
       <c r="U496" t="inlineStr">
         <is>
@@ -77565,13 +77565,13 @@
         </is>
       </c>
       <c r="N502" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="O502" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="R502" t="n">
-        <v>0.09689849618960229</v>
+        <v>0.1085263157323546</v>
       </c>
       <c r="S502" t="inlineStr">
         <is>
@@ -77855,13 +77855,13 @@
         </is>
       </c>
       <c r="N504" t="n">
-        <v>152</v>
+        <v>192</v>
       </c>
       <c r="O504" t="n">
-        <v>152</v>
+        <v>192</v>
       </c>
       <c r="R504" t="n">
-        <v>0.294571428416391</v>
+        <v>0.3720902253680728</v>
       </c>
       <c r="S504" t="inlineStr">
         <is>
@@ -78000,13 +78000,13 @@
         </is>
       </c>
       <c r="N505" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="O505" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="R505" t="n">
-        <v>0.02713157893308864</v>
+        <v>0.03100751878067274</v>
       </c>
       <c r="S505" t="inlineStr">
         <is>
@@ -79077,13 +79077,13 @@
         </is>
       </c>
       <c r="N511" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O511" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R511" t="n">
-        <v>0.007751879695168184</v>
+        <v>0.009689849618960231</v>
       </c>
       <c r="S511" t="inlineStr">
         <is>
@@ -79512,13 +79512,13 @@
         </is>
       </c>
       <c r="N514" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O514" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="R514" t="n">
-        <v>0.01162781954275227</v>
+        <v>0.01937969923792046</v>
       </c>
       <c r="S514" t="inlineStr">
         <is>
@@ -79802,13 +79802,13 @@
         </is>
       </c>
       <c r="N516" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="O516" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="R516" t="n">
-        <v>0.02906954885688069</v>
+        <v>0.03294548870446478</v>
       </c>
       <c r="S516" t="inlineStr">
         <is>
@@ -80092,13 +80092,13 @@
         </is>
       </c>
       <c r="N518" t="n">
-        <v>166</v>
+        <v>246</v>
       </c>
       <c r="O518" t="n">
-        <v>166</v>
+        <v>246</v>
       </c>
       <c r="R518" t="n">
-        <v>0.3217030073494796</v>
+        <v>0.4767406012528433</v>
       </c>
       <c r="S518" t="inlineStr">
         <is>
@@ -80382,13 +80382,13 @@
         </is>
       </c>
       <c r="N520" t="n">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="O520" t="n">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="R520" t="n">
-        <v>0.1220921051988989</v>
+        <v>0.1453477442844034</v>
       </c>
       <c r="S520" t="inlineStr">
         <is>
@@ -80541,10 +80541,10 @@
         </is>
       </c>
       <c r="N521" t="n">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="O521" t="n">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="U521" t="inlineStr">
         <is>
@@ -80920,13 +80920,13 @@
         </is>
       </c>
       <c r="N523" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="O523" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="R523" t="n">
-        <v>0.03488345862825683</v>
+        <v>0.04457330824721705</v>
       </c>
       <c r="S523" t="inlineStr">
         <is>
@@ -81065,13 +81065,13 @@
         </is>
       </c>
       <c r="N524" t="n">
-        <v>158</v>
+        <v>204</v>
       </c>
       <c r="O524" t="n">
-        <v>158</v>
+        <v>204</v>
       </c>
       <c r="R524" t="n">
-        <v>0.3061992479591433</v>
+        <v>0.3953458644535773</v>
       </c>
       <c r="S524" t="inlineStr">
         <is>
@@ -81935,13 +81935,13 @@
         </is>
       </c>
       <c r="N530" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O530" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R530" t="n">
-        <v>0</v>
+        <v>0.001937969923792046</v>
       </c>
       <c r="S530" t="inlineStr">
         <is>
@@ -82225,13 +82225,13 @@
         </is>
       </c>
       <c r="N532" t="n">
-        <v>683</v>
+        <v>828</v>
       </c>
       <c r="O532" t="n">
-        <v>683</v>
+        <v>828</v>
       </c>
       <c r="R532" t="n">
-        <v>1.323633457949967</v>
+        <v>1.604639096899814</v>
       </c>
       <c r="S532" t="inlineStr">
         <is>
@@ -82370,13 +82370,13 @@
         </is>
       </c>
       <c r="N533" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O533" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R533" t="n">
-        <v>0.009689849618960231</v>
+        <v>0.01356578946654432</v>
       </c>
       <c r="S533" t="inlineStr">
         <is>
@@ -83526,13 +83526,13 @@
         </is>
       </c>
       <c r="N541" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O541" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="R541" t="n">
-        <v>0.01937969923792046</v>
+        <v>0.02325563908550455</v>
       </c>
       <c r="S541" t="inlineStr">
         <is>
@@ -83671,13 +83671,13 @@
         </is>
       </c>
       <c r="N542" t="n">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="O542" t="n">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="R542" t="n">
-        <v>0.04069736839963296</v>
+        <v>0.06589097740892956</v>
       </c>
       <c r="S542" t="inlineStr">
         <is>
@@ -84251,13 +84251,13 @@
         </is>
       </c>
       <c r="N546" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="O546" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R546" t="n">
-        <v>0.02131766916171251</v>
+        <v>0.02906954885688069</v>
       </c>
       <c r="S546" t="inlineStr">
         <is>
@@ -87254,13 +87254,13 @@
         </is>
       </c>
       <c r="N566" t="n">
-        <v>2341</v>
+        <v>2729</v>
       </c>
       <c r="O566" t="n">
-        <v>2341</v>
+        <v>2729</v>
       </c>
       <c r="R566" t="n">
-        <v>4.53678759159718</v>
+        <v>5.288719922028493</v>
       </c>
       <c r="S566" t="inlineStr">
         <is>
@@ -87413,10 +87413,10 @@
         </is>
       </c>
       <c r="N567" t="n">
-        <v>2341</v>
+        <v>2729</v>
       </c>
       <c r="O567" t="n">
-        <v>2341</v>
+        <v>2729</v>
       </c>
       <c r="U567" t="inlineStr">
         <is>
@@ -88151,7 +88151,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>75303</v>
+        <v>76048</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-28 02:00:41 UTC
</commit_message>
<xml_diff>
--- a/countries/kr/2026-2029.xlsx
+++ b/countries/kr/2026-2029.xlsx
@@ -56035,13 +56035,13 @@
         </is>
       </c>
       <c r="N362" t="n">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="O362" t="n">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="R362" t="n">
-        <v>0.841078946925748</v>
+        <v>0.844954886773332</v>
       </c>
       <c r="S362" t="inlineStr">
         <is>
@@ -56180,13 +56180,13 @@
         </is>
       </c>
       <c r="N363" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O363" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="R363" t="n">
-        <v>0.1472857142081955</v>
+        <v>0.1453477442844034</v>
       </c>
       <c r="S363" t="inlineStr">
         <is>
@@ -58272,13 +58272,13 @@
         </is>
       </c>
       <c r="N376" t="n">
-        <v>1200</v>
+        <v>1202</v>
       </c>
       <c r="O376" t="n">
-        <v>1200</v>
+        <v>1202</v>
       </c>
       <c r="R376" t="n">
-        <v>2.325563908550455</v>
+        <v>2.329439848398039</v>
       </c>
       <c r="S376" t="inlineStr">
         <is>
@@ -69182,13 +69182,13 @@
         </is>
       </c>
       <c r="N447" t="n">
-        <v>854</v>
+        <v>852</v>
       </c>
       <c r="O447" t="n">
-        <v>854</v>
+        <v>852</v>
       </c>
       <c r="R447" t="n">
-        <v>1.655026314918407</v>
+        <v>1.651150375070823</v>
       </c>
       <c r="S447" t="inlineStr">
         <is>
@@ -70445,13 +70445,13 @@
         </is>
       </c>
       <c r="N455" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O455" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R455" t="n">
-        <v>0.001937969923792046</v>
+        <v>0.003875939847584092</v>
       </c>
       <c r="S455" t="inlineStr">
         <is>
@@ -72761,13 +72761,13 @@
         </is>
       </c>
       <c r="N471" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="O471" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="R471" t="n">
-        <v>0.1821691728364523</v>
+        <v>0.1782932329888682</v>
       </c>
       <c r="S471" t="inlineStr">
         <is>
@@ -73341,13 +73341,13 @@
         </is>
       </c>
       <c r="N475" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="O475" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="R475" t="n">
-        <v>0.2790676690260546</v>
+        <v>0.2810056389498466</v>
       </c>
       <c r="S475" t="inlineStr">
         <is>
@@ -77565,13 +77565,13 @@
         </is>
       </c>
       <c r="N502" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="O502" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="R502" t="n">
-        <v>0.1821691728364523</v>
+        <v>0.1918590224554125</v>
       </c>
       <c r="S502" t="inlineStr">
         <is>
@@ -77855,13 +77855,13 @@
         </is>
       </c>
       <c r="N504" t="n">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="O504" t="n">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="R504" t="n">
-        <v>0.5968947365279502</v>
+        <v>0.6104605259944944</v>
       </c>
       <c r="S504" t="inlineStr">
         <is>
@@ -78000,13 +78000,13 @@
         </is>
       </c>
       <c r="N505" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O505" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R505" t="n">
-        <v>0.0465112781710091</v>
+        <v>0.04844924809480115</v>
       </c>
       <c r="S505" t="inlineStr">
         <is>
@@ -79802,13 +79802,13 @@
         </is>
       </c>
       <c r="N516" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="O516" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="R516" t="n">
-        <v>0.05813909771376138</v>
+        <v>0.06395300748513752</v>
       </c>
       <c r="S516" t="inlineStr">
         <is>
@@ -80092,13 +80092,13 @@
         </is>
       </c>
       <c r="N518" t="n">
-        <v>371</v>
+        <v>398</v>
       </c>
       <c r="O518" t="n">
-        <v>371</v>
+        <v>398</v>
       </c>
       <c r="R518" t="n">
-        <v>0.718986841726849</v>
+        <v>0.7713120296692343</v>
       </c>
       <c r="S518" t="inlineStr">
         <is>
@@ -80382,13 +80382,13 @@
         </is>
       </c>
       <c r="N520" t="n">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="O520" t="n">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="R520" t="n">
-        <v>0.2422462404740058</v>
+        <v>0.2558120299405501</v>
       </c>
       <c r="S520" t="inlineStr">
         <is>
@@ -80541,10 +80541,10 @@
         </is>
       </c>
       <c r="N521" t="n">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="O521" t="n">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="U521" t="inlineStr">
         <is>
@@ -80920,13 +80920,13 @@
         </is>
       </c>
       <c r="N523" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="O523" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="R523" t="n">
-        <v>0.0717048871803057</v>
+        <v>0.07364285710409775</v>
       </c>
       <c r="S523" t="inlineStr">
         <is>
@@ -81065,13 +81065,13 @@
         </is>
       </c>
       <c r="N524" t="n">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="O524" t="n">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="R524" t="n">
-        <v>0.6201503756134548</v>
+        <v>0.6240263154610388</v>
       </c>
       <c r="S524" t="inlineStr">
         <is>
@@ -82225,13 +82225,13 @@
         </is>
       </c>
       <c r="N532" t="n">
-        <v>1308</v>
+        <v>1317</v>
       </c>
       <c r="O532" t="n">
-        <v>1308</v>
+        <v>1317</v>
       </c>
       <c r="R532" t="n">
-        <v>2.534864660319996</v>
+        <v>2.552306389634124</v>
       </c>
       <c r="S532" t="inlineStr">
         <is>
@@ -82370,13 +82370,13 @@
         </is>
       </c>
       <c r="N533" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O533" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="R533" t="n">
-        <v>0.02325563908550455</v>
+        <v>0.02713157893308864</v>
       </c>
       <c r="S533" t="inlineStr">
         <is>
@@ -83526,13 +83526,13 @@
         </is>
       </c>
       <c r="N541" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O541" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="R541" t="n">
-        <v>0.03100751878067274</v>
+        <v>0.03294548870446478</v>
       </c>
       <c r="S541" t="inlineStr">
         <is>
@@ -83671,13 +83671,13 @@
         </is>
       </c>
       <c r="N542" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O542" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="R542" t="n">
-        <v>0.08720864657064206</v>
+        <v>0.09108458641822616</v>
       </c>
       <c r="S542" t="inlineStr">
         <is>
@@ -84106,13 +84106,13 @@
         </is>
       </c>
       <c r="N545" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O545" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R545" t="n">
-        <v>0.007751879695168184</v>
+        <v>0.009689849618960231</v>
       </c>
       <c r="S545" t="inlineStr">
         <is>
@@ -87254,13 +87254,13 @@
         </is>
       </c>
       <c r="N566" t="n">
-        <v>4426</v>
+        <v>4440</v>
       </c>
       <c r="O566" t="n">
-        <v>4426</v>
+        <v>4440</v>
       </c>
       <c r="R566" t="n">
-        <v>8.577454882703595</v>
+        <v>8.604586461636684</v>
       </c>
       <c r="S566" t="inlineStr">
         <is>
@@ -87413,10 +87413,10 @@
         </is>
       </c>
       <c r="N567" t="n">
-        <v>4426</v>
+        <v>4440</v>
       </c>
       <c r="O567" t="n">
-        <v>4426</v>
+        <v>4440</v>
       </c>
       <c r="U567" t="inlineStr">
         <is>
@@ -88151,7 +88151,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>78771</v>
+        <v>78854</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-29 02:06:04 UTC
</commit_message>
<xml_diff>
--- a/countries/kr/2026-2029.xlsx
+++ b/countries/kr/2026-2029.xlsx
@@ -58272,13 +58272,13 @@
         </is>
       </c>
       <c r="N376" t="n">
-        <v>1202</v>
+        <v>1204</v>
       </c>
       <c r="O376" t="n">
-        <v>1202</v>
+        <v>1204</v>
       </c>
       <c r="R376" t="n">
-        <v>2.329439848398039</v>
+        <v>2.333315788245623</v>
       </c>
       <c r="S376" t="inlineStr">
         <is>
@@ -62431,13 +62431,13 @@
         </is>
       </c>
       <c r="N404" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="O404" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="R404" t="n">
-        <v>0.2422462404740058</v>
+        <v>0.2403082705502137</v>
       </c>
       <c r="S404" t="inlineStr">
         <is>
@@ -71315,13 +71315,13 @@
         </is>
       </c>
       <c r="N461" t="n">
-        <v>2512</v>
+        <v>2516</v>
       </c>
       <c r="O461" t="n">
-        <v>2512</v>
+        <v>2516</v>
       </c>
       <c r="R461" t="n">
-        <v>4.86818044856562</v>
+        <v>4.875932328260788</v>
       </c>
       <c r="S461" t="inlineStr">
         <is>
@@ -72761,13 +72761,13 @@
         </is>
       </c>
       <c r="N471" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="O471" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="R471" t="n">
-        <v>0.1782932329888682</v>
+        <v>0.1802312029126603</v>
       </c>
       <c r="S471" t="inlineStr">
         <is>
@@ -73341,13 +73341,13 @@
         </is>
       </c>
       <c r="N475" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O475" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="R475" t="n">
-        <v>0.2810056389498466</v>
+        <v>0.2829436088736387</v>
       </c>
       <c r="S475" t="inlineStr">
         <is>
@@ -74066,13 +74066,13 @@
         </is>
       </c>
       <c r="N480" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O480" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R480" t="n">
-        <v>0.005813909771376137</v>
+        <v>0.007751879695168184</v>
       </c>
       <c r="S480" t="inlineStr">
         <is>
@@ -76344,13 +76344,13 @@
         </is>
       </c>
       <c r="N495" t="n">
-        <v>5538</v>
+        <v>5536</v>
       </c>
       <c r="O495" t="n">
-        <v>5538</v>
+        <v>5536</v>
       </c>
       <c r="R495" t="n">
-        <v>10.73247743796035</v>
+        <v>10.72860149811277</v>
       </c>
       <c r="S495" t="inlineStr">
         <is>
@@ -76503,10 +76503,10 @@
         </is>
       </c>
       <c r="N496" t="n">
-        <v>5538</v>
+        <v>5536</v>
       </c>
       <c r="O496" t="n">
-        <v>5538</v>
+        <v>5536</v>
       </c>
       <c r="U496" t="inlineStr">
         <is>
@@ -77565,13 +77565,13 @@
         </is>
       </c>
       <c r="N502" t="n">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="O502" t="n">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="R502" t="n">
-        <v>0.1918590224554125</v>
+        <v>0.2054248119219569</v>
       </c>
       <c r="S502" t="inlineStr">
         <is>
@@ -77710,13 +77710,13 @@
         </is>
       </c>
       <c r="N503" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="O503" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="R503" t="n">
-        <v>0.007751879695168184</v>
+        <v>0.01744172931412841</v>
       </c>
       <c r="S503" t="inlineStr">
         <is>
@@ -77855,13 +77855,13 @@
         </is>
       </c>
       <c r="N504" t="n">
-        <v>315</v>
+        <v>368</v>
       </c>
       <c r="O504" t="n">
-        <v>315</v>
+        <v>368</v>
       </c>
       <c r="R504" t="n">
-        <v>0.6104605259944944</v>
+        <v>0.7131729319554728</v>
       </c>
       <c r="S504" t="inlineStr">
         <is>
@@ -78000,13 +78000,13 @@
         </is>
       </c>
       <c r="N505" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="O505" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="R505" t="n">
-        <v>0.04844924809480115</v>
+        <v>0.05426315786617728</v>
       </c>
       <c r="S505" t="inlineStr">
         <is>
@@ -79512,13 +79512,13 @@
         </is>
       </c>
       <c r="N514" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="O514" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R514" t="n">
-        <v>0.02906954885688069</v>
+        <v>0.03100751878067274</v>
       </c>
       <c r="S514" t="inlineStr">
         <is>
@@ -79802,13 +79802,13 @@
         </is>
       </c>
       <c r="N516" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="O516" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="R516" t="n">
-        <v>0.06395300748513752</v>
+        <v>0.07751879695168185</v>
       </c>
       <c r="S516" t="inlineStr">
         <is>
@@ -80092,13 +80092,13 @@
         </is>
       </c>
       <c r="N518" t="n">
-        <v>398</v>
+        <v>432</v>
       </c>
       <c r="O518" t="n">
-        <v>398</v>
+        <v>432</v>
       </c>
       <c r="R518" t="n">
-        <v>0.7713120296692343</v>
+        <v>0.8372030070781639</v>
       </c>
       <c r="S518" t="inlineStr">
         <is>
@@ -80382,13 +80382,13 @@
         </is>
       </c>
       <c r="N520" t="n">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="O520" t="n">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="R520" t="n">
-        <v>0.2558120299405501</v>
+        <v>0.2771296991022626</v>
       </c>
       <c r="S520" t="inlineStr">
         <is>
@@ -80541,10 +80541,10 @@
         </is>
       </c>
       <c r="N521" t="n">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="O521" t="n">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="U521" t="inlineStr">
         <is>
@@ -80920,13 +80920,13 @@
         </is>
       </c>
       <c r="N523" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O523" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="R523" t="n">
-        <v>0.07364285710409775</v>
+        <v>0.07558082702788979</v>
       </c>
       <c r="S523" t="inlineStr">
         <is>
@@ -81065,13 +81065,13 @@
         </is>
       </c>
       <c r="N524" t="n">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="O524" t="n">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="R524" t="n">
-        <v>0.6240263154610388</v>
+        <v>0.6530958643179194</v>
       </c>
       <c r="S524" t="inlineStr">
         <is>
@@ -81355,13 +81355,13 @@
         </is>
       </c>
       <c r="N526" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O526" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R526" t="n">
-        <v>0</v>
+        <v>0.001937969923792046</v>
       </c>
       <c r="S526" t="inlineStr">
         <is>
@@ -82225,13 +82225,13 @@
         </is>
       </c>
       <c r="N532" t="n">
-        <v>1317</v>
+        <v>1353</v>
       </c>
       <c r="O532" t="n">
-        <v>1317</v>
+        <v>1353</v>
       </c>
       <c r="R532" t="n">
-        <v>2.552306389634124</v>
+        <v>2.622073306890638</v>
       </c>
       <c r="S532" t="inlineStr">
         <is>
@@ -82370,13 +82370,13 @@
         </is>
       </c>
       <c r="N533" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="O533" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R533" t="n">
-        <v>0.02713157893308864</v>
+        <v>0.02906954885688069</v>
       </c>
       <c r="S533" t="inlineStr">
         <is>
@@ -82515,13 +82515,13 @@
         </is>
       </c>
       <c r="N534" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="O534" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="R534" t="n">
-        <v>0.01937969923792046</v>
+        <v>0.0251936090092966</v>
       </c>
       <c r="S534" t="inlineStr">
         <is>
@@ -83526,13 +83526,13 @@
         </is>
       </c>
       <c r="N541" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="O541" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="R541" t="n">
-        <v>0.03294548870446478</v>
+        <v>0.03875939847584092</v>
       </c>
       <c r="S541" t="inlineStr">
         <is>
@@ -83671,13 +83671,13 @@
         </is>
       </c>
       <c r="N542" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="O542" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="R542" t="n">
-        <v>0.09108458641822616</v>
+        <v>0.09883646611339433</v>
       </c>
       <c r="S542" t="inlineStr">
         <is>
@@ -84251,13 +84251,13 @@
         </is>
       </c>
       <c r="N546" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="O546" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="R546" t="n">
-        <v>0.06007706763755342</v>
+        <v>0.06976691725651366</v>
       </c>
       <c r="S546" t="inlineStr">
         <is>
@@ -84831,13 +84831,13 @@
         </is>
       </c>
       <c r="N550" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O550" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R550" t="n">
-        <v>0</v>
+        <v>0.001937969923792046</v>
       </c>
       <c r="S550" t="inlineStr">
         <is>
@@ -84976,13 +84976,13 @@
         </is>
       </c>
       <c r="N551" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="O551" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="R551" t="n">
-        <v>0.007751879695168184</v>
+        <v>0.01356578946654432</v>
       </c>
       <c r="S551" t="inlineStr">
         <is>
@@ -87254,13 +87254,13 @@
         </is>
       </c>
       <c r="N566" t="n">
-        <v>4440</v>
+        <v>4554</v>
       </c>
       <c r="O566" t="n">
-        <v>4440</v>
+        <v>4554</v>
       </c>
       <c r="R566" t="n">
-        <v>8.604586461636684</v>
+        <v>8.825515032948976</v>
       </c>
       <c r="S566" t="inlineStr">
         <is>
@@ -87413,10 +87413,10 @@
         </is>
       </c>
       <c r="N567" t="n">
-        <v>4440</v>
+        <v>4554</v>
       </c>
       <c r="O567" t="n">
-        <v>4440</v>
+        <v>4554</v>
       </c>
       <c r="U567" t="inlineStr">
         <is>
@@ -88151,7 +88151,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>78854</v>
+        <v>79168</v>
       </c>
     </row>
     <row r="16">

</xml_diff>